<commit_message>
fix plantilla sin formulas
</commit_message>
<xml_diff>
--- a/inventario-backend/plantillas/plantilla_cotizacion.xlsx
+++ b/inventario-backend/plantillas/plantilla_cotizacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FD66A40-B31F-4423-B536-696C7C64A8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0421214-1857-4495-A217-CD299BEFC00B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>INVERSIONES KENOTT SpA</t>
   </si>
@@ -81,12 +81,6 @@
   </si>
   <si>
     <t>TOTAL</t>
-  </si>
-  <si>
-    <t>UNID</t>
-  </si>
-  <si>
-    <t>metros</t>
   </si>
   <si>
     <t>NETO:</t>
@@ -839,495 +833,385 @@
     </row>
     <row r="12" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="16"/>
-      <c r="C12" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C12" s="7"/>
       <c r="D12" s="8"/>
       <c r="E12" s="9"/>
       <c r="F12" s="10"/>
     </row>
     <row r="13" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="17"/>
-      <c r="C13" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C13" s="11"/>
       <c r="D13" s="12"/>
       <c r="E13" s="9"/>
       <c r="F13" s="10"/>
     </row>
     <row r="14" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="16"/>
-      <c r="C14" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C14" s="7"/>
       <c r="D14" s="8"/>
       <c r="E14" s="9"/>
       <c r="F14" s="10"/>
     </row>
     <row r="15" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="17"/>
-      <c r="C15" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C15" s="11"/>
       <c r="D15" s="12"/>
       <c r="E15" s="9"/>
       <c r="F15" s="10"/>
     </row>
     <row r="16" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="16"/>
-      <c r="C16" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C16" s="7"/>
       <c r="D16" s="8"/>
       <c r="E16" s="9"/>
       <c r="F16" s="10"/>
     </row>
     <row r="17" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="17"/>
-      <c r="C17" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C17" s="11"/>
       <c r="D17" s="12"/>
       <c r="E17" s="9"/>
       <c r="F17" s="10"/>
     </row>
     <row r="18" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="16"/>
-      <c r="C18" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C18" s="7"/>
       <c r="D18" s="8"/>
       <c r="E18" s="9"/>
       <c r="F18" s="10"/>
     </row>
     <row r="19" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="17"/>
-      <c r="C19" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C19" s="11"/>
       <c r="D19" s="12"/>
       <c r="E19" s="9"/>
       <c r="F19" s="10"/>
     </row>
     <row r="20" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="16"/>
-      <c r="C20" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C20" s="7"/>
       <c r="D20" s="8"/>
       <c r="E20" s="9"/>
       <c r="F20" s="10"/>
     </row>
     <row r="21" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="17"/>
-      <c r="C21" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C21" s="11"/>
       <c r="D21" s="12"/>
       <c r="E21" s="9"/>
       <c r="F21" s="10"/>
     </row>
     <row r="22" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="16"/>
-      <c r="C22" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C22" s="7"/>
       <c r="D22" s="8"/>
       <c r="E22" s="9"/>
       <c r="F22" s="10"/>
     </row>
     <row r="23" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="17"/>
-      <c r="C23" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C23" s="11"/>
       <c r="D23" s="12"/>
       <c r="E23" s="9"/>
       <c r="F23" s="10"/>
     </row>
     <row r="24" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="16"/>
-      <c r="C24" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C24" s="7"/>
       <c r="D24" s="8"/>
       <c r="E24" s="9"/>
       <c r="F24" s="10"/>
     </row>
     <row r="25" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="17"/>
-      <c r="C25" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C25" s="11"/>
       <c r="D25" s="12"/>
       <c r="E25" s="9"/>
       <c r="F25" s="10"/>
     </row>
     <row r="26" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="16"/>
-      <c r="C26" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C26" s="7"/>
       <c r="D26" s="8"/>
       <c r="E26" s="9"/>
       <c r="F26" s="10"/>
     </row>
     <row r="27" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="17"/>
-      <c r="C27" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C27" s="11"/>
       <c r="D27" s="12"/>
       <c r="E27" s="9"/>
       <c r="F27" s="10"/>
     </row>
     <row r="28" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="16"/>
-      <c r="C28" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C28" s="7"/>
       <c r="D28" s="8"/>
       <c r="E28" s="9"/>
       <c r="F28" s="10"/>
     </row>
     <row r="29" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="17"/>
-      <c r="C29" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C29" s="11"/>
       <c r="D29" s="12"/>
       <c r="E29" s="9"/>
       <c r="F29" s="10"/>
     </row>
     <row r="30" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="16"/>
-      <c r="C30" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C30" s="7"/>
       <c r="D30" s="8"/>
       <c r="E30" s="9"/>
       <c r="F30" s="10"/>
     </row>
     <row r="31" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="17"/>
-      <c r="C31" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C31" s="11"/>
       <c r="D31" s="12"/>
       <c r="E31" s="9"/>
       <c r="F31" s="10"/>
     </row>
     <row r="32" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="16"/>
-      <c r="C32" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C32" s="7"/>
       <c r="D32" s="8"/>
       <c r="E32" s="9"/>
       <c r="F32" s="10"/>
     </row>
     <row r="33" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="17"/>
-      <c r="C33" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C33" s="11"/>
       <c r="D33" s="12"/>
       <c r="E33" s="9"/>
       <c r="F33" s="10"/>
     </row>
     <row r="34" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="16"/>
-      <c r="C34" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C34" s="7"/>
       <c r="D34" s="8"/>
       <c r="E34" s="9"/>
       <c r="F34" s="10"/>
     </row>
     <row r="35" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="17"/>
-      <c r="C35" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C35" s="11"/>
       <c r="D35" s="12"/>
       <c r="E35" s="9"/>
       <c r="F35" s="10"/>
     </row>
     <row r="36" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="16"/>
-      <c r="C36" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C36" s="7"/>
       <c r="D36" s="8"/>
       <c r="E36" s="9"/>
       <c r="F36" s="10"/>
     </row>
     <row r="37" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="17"/>
-      <c r="C37" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C37" s="11"/>
       <c r="D37" s="12"/>
       <c r="E37" s="9"/>
       <c r="F37" s="10"/>
     </row>
     <row r="38" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="16"/>
-      <c r="C38" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C38" s="7"/>
       <c r="D38" s="8"/>
       <c r="E38" s="9"/>
       <c r="F38" s="10"/>
     </row>
     <row r="39" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="17"/>
-      <c r="C39" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C39" s="11"/>
       <c r="D39" s="12"/>
       <c r="E39" s="9"/>
       <c r="F39" s="10"/>
     </row>
     <row r="40" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="16"/>
-      <c r="C40" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C40" s="7"/>
       <c r="D40" s="8"/>
       <c r="E40" s="9"/>
       <c r="F40" s="10"/>
     </row>
     <row r="41" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="17"/>
-      <c r="C41" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C41" s="11"/>
       <c r="D41" s="12"/>
       <c r="E41" s="9"/>
       <c r="F41" s="10"/>
     </row>
     <row r="42" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="16"/>
-      <c r="C42" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C42" s="7"/>
       <c r="D42" s="8"/>
       <c r="E42" s="9"/>
       <c r="F42" s="10"/>
     </row>
     <row r="43" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="17"/>
-      <c r="C43" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C43" s="11"/>
       <c r="D43" s="12"/>
       <c r="E43" s="9"/>
       <c r="F43" s="10"/>
     </row>
     <row r="44" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="16"/>
-      <c r="C44" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C44" s="7"/>
       <c r="D44" s="8"/>
       <c r="E44" s="9"/>
       <c r="F44" s="10"/>
     </row>
     <row r="45" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="17"/>
-      <c r="C45" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C45" s="11"/>
       <c r="D45" s="12"/>
       <c r="E45" s="9"/>
       <c r="F45" s="10"/>
     </row>
     <row r="46" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="16"/>
-      <c r="C46" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C46" s="7"/>
       <c r="D46" s="8"/>
       <c r="E46" s="9"/>
       <c r="F46" s="10"/>
     </row>
     <row r="47" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="17"/>
-      <c r="C47" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C47" s="11"/>
       <c r="D47" s="12"/>
       <c r="E47" s="9"/>
       <c r="F47" s="10"/>
     </row>
     <row r="48" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="16"/>
-      <c r="C48" s="7" t="s">
-        <v>17</v>
-      </c>
+      <c r="C48" s="7"/>
       <c r="D48" s="8"/>
       <c r="E48" s="9"/>
       <c r="F48" s="10"/>
     </row>
     <row r="49" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="17"/>
-      <c r="C49" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C49" s="11"/>
       <c r="D49" s="12"/>
       <c r="E49" s="9"/>
       <c r="F49" s="10"/>
     </row>
     <row r="50" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="16"/>
-      <c r="C50" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C50" s="7"/>
       <c r="D50" s="8"/>
       <c r="E50" s="9"/>
       <c r="F50" s="10"/>
     </row>
     <row r="51" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="17"/>
-      <c r="C51" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C51" s="11"/>
       <c r="D51" s="12"/>
       <c r="E51" s="9"/>
       <c r="F51" s="10"/>
     </row>
     <row r="52" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="16"/>
-      <c r="C52" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C52" s="7"/>
       <c r="D52" s="8"/>
       <c r="E52" s="9"/>
       <c r="F52" s="10"/>
     </row>
     <row r="53" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="17"/>
-      <c r="C53" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C53" s="11"/>
       <c r="D53" s="12"/>
       <c r="E53" s="9"/>
       <c r="F53" s="10"/>
     </row>
     <row r="54" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="16"/>
-      <c r="C54" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C54" s="7"/>
       <c r="D54" s="8"/>
       <c r="E54" s="9"/>
       <c r="F54" s="10"/>
     </row>
     <row r="55" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="17"/>
-      <c r="C55" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C55" s="11"/>
       <c r="D55" s="12"/>
       <c r="E55" s="9"/>
       <c r="F55" s="10"/>
     </row>
     <row r="56" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="16"/>
-      <c r="C56" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C56" s="7"/>
       <c r="D56" s="8"/>
       <c r="E56" s="9"/>
       <c r="F56" s="10"/>
     </row>
     <row r="57" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="17"/>
-      <c r="C57" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C57" s="11"/>
       <c r="D57" s="12"/>
       <c r="E57" s="9"/>
       <c r="F57" s="10"/>
     </row>
     <row r="58" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="16"/>
-      <c r="C58" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C58" s="7"/>
       <c r="D58" s="8"/>
       <c r="E58" s="9"/>
       <c r="F58" s="10"/>
     </row>
     <row r="59" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="17"/>
-      <c r="C59" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C59" s="11"/>
       <c r="D59" s="12"/>
       <c r="E59" s="9"/>
       <c r="F59" s="10"/>
     </row>
     <row r="60" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="16"/>
-      <c r="C60" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C60" s="7"/>
       <c r="D60" s="8"/>
       <c r="E60" s="9"/>
       <c r="F60" s="10"/>
     </row>
     <row r="61" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="17"/>
-      <c r="C61" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C61" s="11"/>
       <c r="D61" s="12"/>
       <c r="E61" s="9"/>
       <c r="F61" s="10"/>
     </row>
     <row r="62" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="16"/>
-      <c r="C62" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C62" s="7"/>
       <c r="D62" s="8"/>
       <c r="E62" s="9"/>
       <c r="F62" s="10"/>
     </row>
     <row r="63" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="17"/>
-      <c r="C63" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C63" s="11"/>
       <c r="D63" s="12"/>
       <c r="E63" s="9"/>
       <c r="F63" s="10"/>
     </row>
     <row r="64" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B64" s="16"/>
-      <c r="C64" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C64" s="7"/>
       <c r="D64" s="8"/>
       <c r="E64" s="9"/>
       <c r="F64" s="10"/>
     </row>
     <row r="65" spans="2:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B65" s="17"/>
-      <c r="C65" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="C65" s="11"/>
       <c r="D65" s="12"/>
       <c r="E65" s="9"/>
       <c r="F65" s="10"/>
     </row>
     <row r="66" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="16"/>
-      <c r="C66" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="C66" s="7"/>
       <c r="D66" s="8"/>
       <c r="E66" s="9"/>
       <c r="F66" s="10"/>
@@ -1340,7 +1224,7 @@
       <c r="C68" s="20"/>
       <c r="D68" s="20"/>
       <c r="E68" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F68" s="13"/>
     </row>
@@ -1349,7 +1233,7 @@
       <c r="C69" s="20"/>
       <c r="D69" s="20"/>
       <c r="E69" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F69" s="13"/>
     </row>
@@ -1358,7 +1242,7 @@
       <c r="C70" s="20"/>
       <c r="D70" s="20"/>
       <c r="E70" s="14" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F70" s="15"/>
     </row>
@@ -1367,7 +1251,7 @@
     </row>
     <row r="72" spans="2:6" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B72" s="23" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C72" s="24"/>
       <c r="D72" s="24"/>

</xml_diff>